<commit_message>
metadata: frictionless datapackage + xlsx fixes
- Add datapackage header subheading in nf1-mouse.org; tangle 6 schema
  blocks into data/metadata_schema.yaml via :tangle directives
- Switch excel sheet selection to dialect.excel.sheet (frictionless v5
  syntax); make paths relative to yaml location
- Reorder mice fields to match xlsx column order (notes, treatment,
  tumor_injection_date)
- Populate mice.sex='f' for all 140 rows (per DoD Narrative 2024-10-09)
- Fix 15 samples.collection_date cells (tab-prefixed M/D/YYYY -> ISO;
  unknown-date annotation -> blank)

Validates clean with: frictionless validate --type package
data/metadata_schema.yaml --schema-sync
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -21,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,13 +63,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,6 +517,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>washu</t>
@@ -552,6 +559,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>washu</t>
@@ -589,6 +601,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>washu</t>
@@ -626,6 +643,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>washu</t>
@@ -663,6 +685,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>washu</t>
@@ -700,6 +727,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>washu</t>
@@ -737,6 +769,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>washu</t>
@@ -774,6 +811,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>washu</t>
@@ -811,6 +853,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>washu</t>
@@ -848,6 +895,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>washu</t>
@@ -885,6 +937,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>washu</t>
@@ -922,6 +979,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>washu</t>
@@ -959,6 +1021,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>washu</t>
@@ -996,6 +1063,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1033,6 +1105,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1070,6 +1147,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1107,6 +1189,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1144,6 +1231,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1181,6 +1273,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1218,6 +1315,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1255,6 +1357,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1292,6 +1399,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1329,6 +1441,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1366,6 +1483,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1403,6 +1525,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1440,6 +1567,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1477,6 +1609,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1514,6 +1651,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1551,6 +1693,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1588,6 +1735,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1625,6 +1777,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1662,6 +1819,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1699,6 +1861,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1736,6 +1903,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1773,6 +1945,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1810,6 +1987,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1847,6 +2029,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1884,6 +2071,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1921,6 +2113,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1958,6 +2155,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>washu</t>
@@ -1995,6 +2197,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2032,6 +2239,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2069,6 +2281,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2106,6 +2323,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2143,6 +2365,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2180,6 +2407,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2217,6 +2449,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2254,6 +2491,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2291,6 +2533,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2323,6 +2570,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2360,6 +2612,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2397,6 +2654,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2434,6 +2696,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2471,6 +2738,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2503,6 +2775,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2535,6 +2812,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2567,6 +2849,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2604,6 +2891,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2641,6 +2933,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2673,6 +2970,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2710,6 +3012,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2747,6 +3054,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2784,6 +3096,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F64" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2821,6 +3138,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2858,6 +3180,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2895,6 +3222,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2927,6 +3259,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2959,6 +3296,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>washu</t>
@@ -2991,6 +3333,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3023,6 +3370,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3055,6 +3407,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3087,6 +3444,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3119,6 +3481,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3151,6 +3518,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3183,6 +3555,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3215,6 +3592,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3247,6 +3629,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3284,6 +3671,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3321,6 +3713,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3358,6 +3755,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3395,6 +3797,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3432,6 +3839,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3469,6 +3881,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3506,6 +3923,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3543,6 +3965,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3580,6 +4007,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3617,6 +4049,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3654,6 +4091,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3691,6 +4133,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3728,6 +4175,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3765,6 +4217,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3802,6 +4259,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3839,6 +4301,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3876,6 +4343,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3913,6 +4385,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3950,6 +4427,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr">
         <is>
           <t>washu</t>
@@ -3987,6 +4469,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4024,6 +4511,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4061,6 +4553,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4098,6 +4595,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4135,6 +4637,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F102" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4172,6 +4679,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F103" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4209,6 +4721,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4246,6 +4763,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F105" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4283,6 +4805,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F106" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4320,6 +4847,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F107" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4357,6 +4889,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F108" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4394,6 +4931,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4431,6 +4973,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4468,6 +5015,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F111" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4505,6 +5057,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F112" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4542,6 +5099,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F113" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4574,6 +5136,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F114" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4611,6 +5178,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F115" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4648,6 +5220,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F116" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4685,6 +5262,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F117" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4717,6 +5299,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F118" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4754,6 +5341,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F119" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4786,6 +5378,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F120" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4818,6 +5415,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F121" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4850,6 +5452,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F122" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4882,6 +5489,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F123" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4914,6 +5526,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F124" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4951,6 +5568,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F125" t="inlineStr">
         <is>
           <t>washu</t>
@@ -4983,6 +5605,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F126" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5015,6 +5642,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F127" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5052,6 +5684,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F128" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5089,6 +5726,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F129" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5126,6 +5768,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F130" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5163,6 +5810,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F131" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5195,6 +5847,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F132" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5232,6 +5889,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F133" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5264,6 +5926,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F134" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5301,6 +5968,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5333,6 +6005,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F136" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5370,6 +6047,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5407,6 +6089,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5444,6 +6131,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F139" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5481,6 +6173,11 @@
           <t>nod_cg_rag1_null_il2rg_null</t>
         </is>
       </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
       <c r="F140" t="inlineStr">
         <is>
           <t>washu</t>
@@ -5516,6 +6213,11 @@
       <c r="C141" t="inlineStr">
         <is>
           <t>nod_cg_rag1_null_il2rg_null</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>f</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -6739,11 +7441,6 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>? - likely on tube</t>
-        </is>
-      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>new -80, Rack 7, row B, column 2</t>
@@ -7166,10 +7863,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E52" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -7193,10 +7888,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E53" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -7220,10 +7913,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E54" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -7247,10 +7938,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E55" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -7274,10 +7963,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E56" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -7301,10 +7988,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E57" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -7328,10 +8013,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/17/2024</t>
-        </is>
+      <c r="E58" s="4" t="n">
+        <v>45490</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -7355,10 +8038,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E59" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -7382,10 +8063,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E60" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -7409,10 +8088,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E61" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -7436,10 +8113,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E62" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -7463,10 +8138,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E63" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -7490,10 +8163,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E64" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -7517,10 +8188,8 @@
           <t>terminal</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	7/6/2024</t>
-        </is>
+      <c r="E65" s="4" t="n">
+        <v>45479</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
metadata: ingest sample volumes from NCI murine/human manifest
Populate samples.volume_ul for 30 mouse samples from the
Murine_Human Plasma Sample NCI Manifest.xlsx source file.
Matched by mouse_id (via alt_subj) × collection_date × bleed_type;
all 30 matched uniquely. Human rows in the manifest (25) skipped.
Normalized manifest shorthand '2-055 X-Y' -> 'JH-2-055 X-Y'.
Package still validates clean.
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -6471,6 +6471,9 @@
           <t>2024-08-20</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>450</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>nf1_lib95</t>
@@ -6503,6 +6506,9 @@
           <t>2024-08-20</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>500</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>nf1_lib96</t>
@@ -6535,6 +6541,9 @@
           <t>2024-08-20</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>450</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>nf1_lib97</t>
@@ -6567,6 +6576,9 @@
           <t>2024-08-30</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v>500</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>nf1_lib98</t>
@@ -6599,6 +6611,9 @@
           <t>2024-08-30</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v>400</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>nf1_lib99</t>
@@ -6631,6 +6646,9 @@
           <t>2024-08-30</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v>400</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>nf1_lib100</t>
@@ -6663,6 +6681,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>50</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t xml:space="preserve">nf1_lib101; m13 JH-2-005 1-4 D19 S </t>
@@ -6695,6 +6716,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>50</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>nf1_lib102; m14 JH-2-005 4-5 D19 S</t>
@@ -6727,6 +6751,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>50</v>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>nf1_lib103; m15 JH-2-005 5-5 D19 S</t>
@@ -6759,6 +6786,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>50</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>nf1_lib104; m16 JH-2-005 3-2 D19 S</t>
@@ -6791,6 +6821,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F12" t="n">
+        <v>50</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>nf1_lib105; m17 JH-2-005 3-3 D19 S</t>
@@ -6823,6 +6856,9 @@
           <t>2024-10-01</t>
         </is>
       </c>
+      <c r="F13" t="n">
+        <v>50</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>nf1_lib106; m18 JH-2-005 7-5 D19 S</t>
@@ -6855,6 +6891,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F14" t="n">
+        <v>50</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>nf1_lib107</t>
@@ -6887,6 +6926,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>nf1_lib108</t>
@@ -6919,6 +6961,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F16" t="n">
+        <v>50</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>nf1_lib109</t>
@@ -6951,6 +6996,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>nf1_lib110</t>
@@ -6983,6 +7031,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F18" t="n">
+        <v>50</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>nf1_lib111</t>
@@ -7015,6 +7066,9 @@
           <t>2024-10-29</t>
         </is>
       </c>
+      <c r="F19" t="n">
+        <v>50</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>nf1_lib112</t>
@@ -7047,6 +7101,9 @@
           <t>2024-06-05</t>
         </is>
       </c>
+      <c r="F20" t="n">
+        <v>400</v>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>mouse terminal bleed 400 ul</t>
@@ -7074,6 +7131,9 @@
           <t>2024-06-05</t>
         </is>
       </c>
+      <c r="F21" t="n">
+        <v>300</v>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>mouse terminal bleed 300 ul</t>
@@ -7101,6 +7161,9 @@
           <t>2024-06-05</t>
         </is>
       </c>
+      <c r="F22" t="n">
+        <v>300</v>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>mouse terminal bleed 300 ul</t>
@@ -7128,6 +7191,9 @@
           <t>2024-06-12</t>
         </is>
       </c>
+      <c r="F23" t="n">
+        <v>400</v>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>mouse terminal bleed 400 ul</t>
@@ -7155,6 +7221,9 @@
           <t>2024-06-12</t>
         </is>
       </c>
+      <c r="F24" t="n">
+        <v>400</v>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>mouse terminal bleed 400 ul</t>
@@ -7182,6 +7251,9 @@
           <t>2024-06-12</t>
         </is>
       </c>
+      <c r="F25" t="n">
+        <v>400</v>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>mouse terminal bleed 400 ul</t>
@@ -7209,6 +7281,9 @@
           <t>2024-09-17</t>
         </is>
       </c>
+      <c r="F26" t="n">
+        <v>50</v>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>mouse serial bleed</t>
@@ -7236,6 +7311,9 @@
           <t>2024-09-17</t>
         </is>
       </c>
+      <c r="F27" t="n">
+        <v>50</v>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>mouse serial bleed</t>
@@ -7263,6 +7341,9 @@
           <t>2024-09-17</t>
         </is>
       </c>
+      <c r="F28" t="n">
+        <v>50</v>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>mouse serial bleed</t>
@@ -7290,6 +7371,9 @@
           <t>2024-10-22</t>
         </is>
       </c>
+      <c r="F29" t="n">
+        <v>50</v>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>mouse serial bleed</t>
@@ -7317,6 +7401,9 @@
           <t>2024-10-22</t>
         </is>
       </c>
+      <c r="F30" t="n">
+        <v>50</v>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>mouse serial bleed</t>
@@ -7343,6 +7430,9 @@
         <is>
           <t>2024-10-22</t>
         </is>
+      </c>
+      <c r="F31" t="n">
+        <v>50</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
metadata: add tumor_injection_site field to mice schema
Adds optional enum field (flank, sciatic_nerve, intramuscular,
subcutaneous, other) to the mice sheet. Column created empty —
injection site data not available from source records.
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:M141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,6 +498,11 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>tumor_injection_date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>tumor_injection_site</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
metadata: add pdx_lines.donor_sex; resolve 3 of 6 lines
Adds optional donor_sex enum (m/f) to pdx_lines schema. Populated
WU-225, WU-356, WU-487 as male from Sarcoma Banking Subjects List
(WashU). Added TODO heading naming JH-2-002, JH-2-055, MN2 as
pending Hirbe/Pratilas lab confirmation.

Motivation: all 140 host mice are female, so Y-chromosome cfDNA in
samples from male-donor-PDX mice = tumor fraction cross-check.
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -6257,7 +6257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6281,6 +6281,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>donor_sex</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6315,6 +6320,11 @@
           <t>washu</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6349,6 +6359,11 @@
           <t>washu</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6391,6 +6406,11 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>Chr8q gain per Hirbe email Nov 2024</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
     </row>

</xml_diff>